<commit_message>
[auto-snapshot] 2026-04-26 08:00 | onda-hompage | 44 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_nail/영등포_네일샵.xlsx
+++ b/naver-place-crawler/results_nail/영등포_네일샵.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V184"/>
+  <dimension ref="A1:V205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17618,6 +17618,1940 @@
         </is>
       </c>
     </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>ROXY NAIL</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr"/>
+      <c r="D185" t="inlineStr"/>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>0507-1493-7677</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 당산로 100 1층 록시네일</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>http://Instagram.com/roxynail_</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr"/>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P185" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q185" t="n">
+        <v>8</v>
+      </c>
+      <c r="R185" t="n">
+        <v>35</v>
+      </c>
+      <c r="S185" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>36104695</t>
+        </is>
+      </c>
+      <c r="U185" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/36104695</t>
+        </is>
+      </c>
+      <c r="V185" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>유벨네일</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr"/>
+      <c r="D186" t="inlineStr"/>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>0507-1318-4266</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 영신로 238 2층 206호</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_xmyHUn</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr"/>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P186" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q186" t="n">
+        <v>8</v>
+      </c>
+      <c r="R186" t="n">
+        <v>52</v>
+      </c>
+      <c r="S186" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>2042628410</t>
+        </is>
+      </c>
+      <c r="U186" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2042628410</t>
+        </is>
+      </c>
+      <c r="V186" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>네일보나</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>yunyue499@naver.com</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr"/>
+      <c r="E187" t="inlineStr"/>
+      <c r="F187" t="inlineStr"/>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 도림로54길 7 1층 네일보나</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_tTmpT/chat</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr"/>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P187" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q187" t="n">
+        <v>1</v>
+      </c>
+      <c r="R187" t="n">
+        <v>17</v>
+      </c>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>1043256456</t>
+        </is>
+      </c>
+      <c r="U187" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1043256456</t>
+        </is>
+      </c>
+      <c r="V187" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>마틸다네일M 여의도점</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>vin2roo@naver.com</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr"/>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>0507-1437-3082</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 국제금융로 78 홍우빌딩 1003호</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/matilda_nailshop</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr"/>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P188" t="n">
+        <v>137</v>
+      </c>
+      <c r="Q188" t="n">
+        <v>36</v>
+      </c>
+      <c r="R188" t="n">
+        <v>173</v>
+      </c>
+      <c r="S188" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>1556640253</t>
+        </is>
+      </c>
+      <c r="U188" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1556640253</t>
+        </is>
+      </c>
+      <c r="V188" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>NailZizi</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr"/>
+      <c r="D189" t="inlineStr"/>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>0507-1314-6188</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr"/>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 가마산로63길 10-6 1층 네일지지</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_msexcb</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr"/>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P189" t="n">
+        <v>133</v>
+      </c>
+      <c r="Q189" t="n">
+        <v>28</v>
+      </c>
+      <c r="R189" t="n">
+        <v>161</v>
+      </c>
+      <c r="S189" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T189" t="inlineStr">
+        <is>
+          <t>1934965398</t>
+        </is>
+      </c>
+      <c r="U189" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1934965398</t>
+        </is>
+      </c>
+      <c r="V189" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>네일올리브</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>reyia@naver.com</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr"/>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>0507-1401-6151</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 양평로22길 12 1층</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>http://instagram.com/nailolive_seonyudo</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr"/>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P190" t="n">
+        <v>402</v>
+      </c>
+      <c r="Q190" t="n">
+        <v>43</v>
+      </c>
+      <c r="R190" t="n">
+        <v>445</v>
+      </c>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>37642650</t>
+        </is>
+      </c>
+      <c r="U190" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/37642650</t>
+        </is>
+      </c>
+      <c r="V190" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>디오네일.THE O NAIL</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>armanio@naver.com</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr"/>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>02-2676-6311</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 당산로 222 당산디오빌 지하1층 114호</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr"/>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P191" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q191" t="n">
+        <v>0</v>
+      </c>
+      <c r="R191" t="n">
+        <v>7</v>
+      </c>
+      <c r="S191" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T191" t="inlineStr">
+        <is>
+          <t>32333026</t>
+        </is>
+      </c>
+      <c r="U191" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/32333026</t>
+        </is>
+      </c>
+      <c r="V191" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>더퀸네일</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>mimvely_j@naver.com</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr"/>
+      <c r="E192" t="inlineStr"/>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 당산로 47 2층 더퀸네일</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/mimvely_j</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr"/>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P192" t="n">
+        <v>257</v>
+      </c>
+      <c r="Q192" t="n">
+        <v>166</v>
+      </c>
+      <c r="R192" t="n">
+        <v>423</v>
+      </c>
+      <c r="S192" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T192" t="inlineStr">
+        <is>
+          <t>1355193331</t>
+        </is>
+      </c>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1355193331</t>
+        </is>
+      </c>
+      <c r="V192" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>금붕어네일 여의도점</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>ilikepotatopizza@naver.com</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr"/>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>0507-1389-8486</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 국제금융로6길 30 백상빌딩 411호 금붕어네일</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/goldfish.nail</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr"/>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P193" t="n">
+        <v>659</v>
+      </c>
+      <c r="Q193" t="n">
+        <v>216</v>
+      </c>
+      <c r="R193" t="n">
+        <v>875</v>
+      </c>
+      <c r="S193" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>1184687193</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1184687193</t>
+        </is>
+      </c>
+      <c r="V193" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>예민네일</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>daonnail0305@naver.com</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr"/>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>0507-1324-5290</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 여의대방로35길 40 1층 예민네일</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>https://open.kakao.com/o/sXdZmmTg</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr"/>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P194" t="n">
+        <v>341</v>
+      </c>
+      <c r="Q194" t="n">
+        <v>2</v>
+      </c>
+      <c r="R194" t="n">
+        <v>343</v>
+      </c>
+      <c r="S194" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T194" t="inlineStr">
+        <is>
+          <t>1128888555</t>
+        </is>
+      </c>
+      <c r="U194" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1128888555</t>
+        </is>
+      </c>
+      <c r="V194" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>네일은 문래</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr"/>
+      <c r="D195" t="inlineStr"/>
+      <c r="E195" t="inlineStr"/>
+      <c r="F195" t="inlineStr"/>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 문래로 84 상가동 105호 네일은</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>https://pf.kakao.com/_UfxdRb</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr"/>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P195" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q195" t="n">
+        <v>12</v>
+      </c>
+      <c r="R195" t="n">
+        <v>92</v>
+      </c>
+      <c r="S195" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T195" t="inlineStr">
+        <is>
+          <t>1843875225</t>
+        </is>
+      </c>
+      <c r="U195" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1843875225</t>
+        </is>
+      </c>
+      <c r="V195" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>수다네일 서울1호점</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>hsleek925@naver.com</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr"/>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>02-2068-2046</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr"/>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 당산로 159</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr"/>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P196" t="n">
+        <v>97</v>
+      </c>
+      <c r="Q196" t="n">
+        <v>3</v>
+      </c>
+      <c r="R196" t="n">
+        <v>100</v>
+      </c>
+      <c r="S196" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T196" t="inlineStr">
+        <is>
+          <t>36105141</t>
+        </is>
+      </c>
+      <c r="U196" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/36105141</t>
+        </is>
+      </c>
+      <c r="V196" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>네일랄라</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>lalla-nail@naver.com</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr"/>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>02-761-6130</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr"/>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 국제금융로 70 1층 112호</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/lalla-nail</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr"/>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P197" t="n">
+        <v>413</v>
+      </c>
+      <c r="Q197" t="n">
+        <v>156</v>
+      </c>
+      <c r="R197" t="n">
+        <v>569</v>
+      </c>
+      <c r="S197" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>1694954156</t>
+        </is>
+      </c>
+      <c r="U197" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1694954156</t>
+        </is>
+      </c>
+      <c r="V197" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>유니뷰티랩</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>nuri0331@naver.com</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr"/>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>0507-1320-1714</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr"/>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 국회대로54길 10 상가13동 102호(영등포동7가, 아 크로타워 스퀘어)</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/u_nibeautylab</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr"/>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P198" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q198" t="n">
+        <v>30</v>
+      </c>
+      <c r="R198" t="n">
+        <v>80</v>
+      </c>
+      <c r="S198" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>1224258897</t>
+        </is>
+      </c>
+      <c r="U198" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1224258897</t>
+        </is>
+      </c>
+      <c r="V198" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>네일포유</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>nail_for_u@naver.com</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr"/>
+      <c r="E199" t="inlineStr"/>
+      <c r="F199" t="inlineStr"/>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 의사당대로 166 9호선 샛강역 지하 상가</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr"/>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P199" t="n">
+        <v>49</v>
+      </c>
+      <c r="Q199" t="n">
+        <v>1</v>
+      </c>
+      <c r="R199" t="n">
+        <v>50</v>
+      </c>
+      <c r="S199" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>1198739781</t>
+        </is>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1198739781</t>
+        </is>
+      </c>
+      <c r="V199" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>네일스토리</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>yeju0414@naver.com</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr"/>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>0507-1370-8734</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 디지털로 353 1층 네일스토리</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr"/>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P200" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q200" t="n">
+        <v>12</v>
+      </c>
+      <c r="R200" t="n">
+        <v>23</v>
+      </c>
+      <c r="S200" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T200" t="inlineStr">
+        <is>
+          <t>79673372</t>
+        </is>
+      </c>
+      <c r="U200" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/79673372</t>
+        </is>
+      </c>
+      <c r="V200" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>찹쌀 네일</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>daonnail0305@naver.com</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr"/>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>0507-1317-5004</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 국회대로50길 20 상가동 2층 227호</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/cabssalneil?igsh=Mzlna2d0Z2VzdzRr&amp;utm_source=ig_contact_invite</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr"/>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P201" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q201" t="n">
+        <v>0</v>
+      </c>
+      <c r="R201" t="n">
+        <v>3</v>
+      </c>
+      <c r="S201" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T201" t="inlineStr">
+        <is>
+          <t>2095561893</t>
+        </is>
+      </c>
+      <c r="U201" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2095561893</t>
+        </is>
+      </c>
+      <c r="V201" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>네일은</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr"/>
+      <c r="D202" t="inlineStr"/>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>02-6013-8231</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr"/>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>서울특별시 동작구 여의대방로 188-1 1층</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/naileun8231</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr"/>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P202" t="n">
+        <v>34</v>
+      </c>
+      <c r="Q202" t="n">
+        <v>9</v>
+      </c>
+      <c r="R202" t="n">
+        <v>43</v>
+      </c>
+      <c r="S202" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>1943789782</t>
+        </is>
+      </c>
+      <c r="U202" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1943789782</t>
+        </is>
+      </c>
+      <c r="V202" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>네일 오운페이스</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>bongbong323@naver.com</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr"/>
+      <c r="E203" t="inlineStr"/>
+      <c r="F203" t="inlineStr"/>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 도림로139길 4 대신빌딩 203호</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nail.ownpace</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr"/>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P203" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q203" t="n">
+        <v>12</v>
+      </c>
+      <c r="R203" t="n">
+        <v>52</v>
+      </c>
+      <c r="S203" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T203" t="inlineStr">
+        <is>
+          <t>1158657633</t>
+        </is>
+      </c>
+      <c r="U203" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1158657633</t>
+        </is>
+      </c>
+      <c r="V203" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>미하루뷰티</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>fbtn2917@naver.com</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr"/>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>0507-1485-5188</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr"/>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 대림로27나길 14 1층</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr"/>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P204" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q204" t="n">
+        <v>0</v>
+      </c>
+      <c r="R204" t="n">
+        <v>8</v>
+      </c>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>2016346574</t>
+        </is>
+      </c>
+      <c r="U204" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2016346574</t>
+        </is>
+      </c>
+      <c r="V204" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>향네일</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>ekgid9405@naver.com</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr"/>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>02-831-9168</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr"/>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>서울특별시 영등포구 도신로64길 14 1F</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr"/>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P205" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q205" t="n">
+        <v>1</v>
+      </c>
+      <c r="R205" t="n">
+        <v>5</v>
+      </c>
+      <c r="S205" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>1278016908</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1278016908</t>
+        </is>
+      </c>
+      <c r="V205" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>